<commit_message>
chore(daily): 自动更新 data.js + stock_data.xlsx (北京时间 2026-09-10 03:01)
</commit_message>
<xml_diff>
--- a/stock_data.xlsx
+++ b/stock_data.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L485"/>
+  <dimension ref="A1:L486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20803,6 +20803,48 @@
       </c>
       <c r="L485" t="n">
         <v>-0.01188932122784259</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>600276.SH</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="D486" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="E486" t="n">
+        <v>44.64</v>
+      </c>
+      <c r="F486" t="n">
+        <v>44.71</v>
+      </c>
+      <c r="G486" t="n">
+        <v>45.71</v>
+      </c>
+      <c r="H486" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I486" t="n">
+        <v>-2.19</v>
+      </c>
+      <c r="J486" t="n">
+        <v>716944</v>
+      </c>
+      <c r="K486" t="n">
+        <v>3214392264</v>
+      </c>
+      <c r="L486" t="n">
+        <v>-0.02187705097352877</v>
       </c>
     </row>
   </sheetData>
@@ -20816,7 +20858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L485"/>
+  <dimension ref="A1:L486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41203,6 +41245,48 @@
       </c>
       <c r="L485" t="n">
         <v>-0.01188932122784259</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>600276.SH</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="D486" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="E486" t="n">
+        <v>44.64</v>
+      </c>
+      <c r="F486" t="n">
+        <v>44.71</v>
+      </c>
+      <c r="G486" t="n">
+        <v>45.71</v>
+      </c>
+      <c r="H486" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I486" t="n">
+        <v>-2.19</v>
+      </c>
+      <c r="J486" t="n">
+        <v>716944</v>
+      </c>
+      <c r="K486" t="n">
+        <v>3214392264</v>
+      </c>
+      <c r="L486" t="n">
+        <v>-0.02187705097352877</v>
       </c>
     </row>
   </sheetData>
@@ -41216,7 +41300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L485"/>
+  <dimension ref="A1:L486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61603,6 +61687,48 @@
       </c>
       <c r="L485" t="n">
         <v>0.006837606837606813</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>000001.SZ</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="D486" t="n">
+        <v>11.79</v>
+      </c>
+      <c r="E486" t="n">
+        <v>11.69</v>
+      </c>
+      <c r="F486" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G486" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="H486" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="I486" t="n">
+        <v>-0.68</v>
+      </c>
+      <c r="J486" t="n">
+        <v>582306</v>
+      </c>
+      <c r="K486" t="n">
+        <v>682946782.66</v>
+      </c>
+      <c r="L486" t="n">
+        <v>-0.006791171477079749</v>
       </c>
     </row>
   </sheetData>
@@ -61616,7 +61742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L485"/>
+  <dimension ref="A1:L486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82005,6 +82131,48 @@
         <v>0.006837606837606813</v>
       </c>
     </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>000001.SZ</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="D486" t="n">
+        <v>11.79</v>
+      </c>
+      <c r="E486" t="n">
+        <v>11.69</v>
+      </c>
+      <c r="F486" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G486" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="H486" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="I486" t="n">
+        <v>-0.68</v>
+      </c>
+      <c r="J486" t="n">
+        <v>582306</v>
+      </c>
+      <c r="K486" t="n">
+        <v>682946782.66</v>
+      </c>
+      <c r="L486" t="n">
+        <v>-0.006791171477079749</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(daily): 自动更新 data.js + stock_data.xlsx (北京时间 2026-10-09 04:59)
</commit_message>
<xml_diff>
--- a/stock_data.xlsx
+++ b/stock_data.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L486"/>
+  <dimension ref="A1:L487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20841,6 +20841,48 @@
       </c>
       <c r="L486" t="n">
         <v>0.03463393248575208</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>600276.SH</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="D487" t="n">
+        <v>47.58</v>
+      </c>
+      <c r="E487" t="n">
+        <v>46.24</v>
+      </c>
+      <c r="F487" t="n">
+        <v>47.01</v>
+      </c>
+      <c r="G487" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="H487" t="n">
+        <v>-0.1900000000000048</v>
+      </c>
+      <c r="I487" t="n">
+        <v>-0.4025423728813661</v>
+      </c>
+      <c r="J487" t="n">
+        <v>77046704</v>
+      </c>
+      <c r="K487" t="n">
+        <v>3629285000</v>
+      </c>
+      <c r="L487" t="n">
+        <v>-0.004025423728813649</v>
       </c>
     </row>
   </sheetData>
@@ -20854,7 +20896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L486"/>
+  <dimension ref="A1:L487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41279,6 +41321,48 @@
       </c>
       <c r="L486" t="n">
         <v>0.03463393248575208</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>600276.SH</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="D487" t="n">
+        <v>47.58</v>
+      </c>
+      <c r="E487" t="n">
+        <v>46.24</v>
+      </c>
+      <c r="F487" t="n">
+        <v>47.01</v>
+      </c>
+      <c r="G487" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="H487" t="n">
+        <v>-0.1900000000000048</v>
+      </c>
+      <c r="I487" t="n">
+        <v>-0.4025423728813661</v>
+      </c>
+      <c r="J487" t="n">
+        <v>77046704</v>
+      </c>
+      <c r="K487" t="n">
+        <v>3629285000</v>
+      </c>
+      <c r="L487" t="n">
+        <v>-0.004025423728813649</v>
       </c>
     </row>
   </sheetData>
@@ -41292,7 +41376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L486"/>
+  <dimension ref="A1:L487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61717,6 +61801,48 @@
       </c>
       <c r="L486" t="n">
         <v>0.01938325991189438</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>000001.SZ</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="D487" t="n">
+        <v>11.87</v>
+      </c>
+      <c r="E487" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="F487" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="G487" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="H487" t="n">
+        <v>0.2099999999999991</v>
+      </c>
+      <c r="I487" t="n">
+        <v>1.815038893690571</v>
+      </c>
+      <c r="J487" t="n">
+        <v>149327837</v>
+      </c>
+      <c r="K487" t="n">
+        <v>1743402500</v>
+      </c>
+      <c r="L487" t="n">
+        <v>0.01815038893690568</v>
       </c>
     </row>
   </sheetData>
@@ -61730,7 +61856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L486"/>
+  <dimension ref="A1:L487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82157,6 +82283,48 @@
         <v>0.01938325991189438</v>
       </c>
     </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>000001.SZ</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="D487" t="n">
+        <v>11.87</v>
+      </c>
+      <c r="E487" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="F487" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="G487" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="H487" t="n">
+        <v>0.2099999999999991</v>
+      </c>
+      <c r="I487" t="n">
+        <v>1.815038893690571</v>
+      </c>
+      <c r="J487" t="n">
+        <v>149327837</v>
+      </c>
+      <c r="K487" t="n">
+        <v>1743402500</v>
+      </c>
+      <c r="L487" t="n">
+        <v>0.01815038893690568</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>